<commit_message>
Add EMERGING-E support and parser path autodetection
</commit_message>
<xml_diff>
--- a/mario/test/supporting_files/add_sector_iot_inventories_filled.xlsx
+++ b/mario/test/supporting_files/add_sector_iot_inventories_filled.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzorinaldi/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzorinaldi/Documents/GitHub/MARIO/mario/test/supporting_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C138145D-4327-E54C-8816-68259D458F06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A155198-E7D0-A44E-A386-C30D85D777BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="10420" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -24,12 +24,25 @@
     <sheet name="new_ind" sheetId="9" r:id="rId9"/>
     <sheet name="new_ser" sheetId="10" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="57">
   <si>
     <t>Region</t>
   </si>
@@ -197,6 +210,9 @@
   </si>
   <si>
     <t>All</t>
+  </si>
+  <si>
+    <t>Split</t>
   </si>
 </sst>
 </file>
@@ -295,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -310,6 +326,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -683,6 +700,12 @@
       <c r="E2" t="s">
         <v>15</v>
       </c>
+      <c r="H2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -988,8 +1011,16 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -1009,6 +1040,42 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2">
+        <f>0.05*53115504</f>
+        <v>2655775.2000000002</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="6">
+        <f>0.05*1195683</f>
+        <v>59784.15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1018,8 +1085,16 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -1042,6 +1117,48 @@
       </c>
       <c r="G1" s="1" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="6">
+        <f>0.05*288442</f>
+        <v>14422.1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3">
+        <f>0.05*437620</f>
+        <v>21881</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1053,6 +1170,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="3" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">

</xml_diff>